<commit_message>
Add func to merge on isin
</commit_message>
<xml_diff>
--- a/off-disc/bank-nifty-ffat.xlsx
+++ b/off-disc/bank-nifty-ffat.xlsx
@@ -471,7 +471,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>ticker</t>
+          <t>symbol</t>
         </is>
       </c>
     </row>
@@ -500,17 +500,9 @@
       <c r="F2" t="n">
         <v>28.49</v>
       </c>
-      <c r="G2" t="n">
-        <v>21.15</v>
-      </c>
-      <c r="H2" t="n">
-        <v>45.96</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>NSE:HDFCBANK</t>
-        </is>
-      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -537,17 +529,9 @@
       <c r="F3" t="n">
         <v>24.38</v>
       </c>
-      <c r="G3" t="n">
-        <v>18.73</v>
-      </c>
-      <c r="H3" t="n">
-        <v>73.59999999999999</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>NSE:ICICIBANK</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -574,17 +558,9 @@
       <c r="F4" t="n">
         <v>9.17</v>
       </c>
-      <c r="G4" t="n">
-        <v>9.859999999999999</v>
-      </c>
-      <c r="H4" t="n">
-        <v>89.01000000000001</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>NSE:SBIN</t>
-        </is>
-      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -611,17 +587,9 @@
       <c r="F5" t="n">
         <v>8.960000000000001</v>
       </c>
-      <c r="G5" t="n">
-        <v>22.17</v>
-      </c>
-      <c r="H5" t="n">
-        <v>96.31</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>NSE:KOTAKBANK</t>
-        </is>
-      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -648,17 +616,9 @@
       <c r="F6" t="n">
         <v>8.779999999999999</v>
       </c>
-      <c r="G6" t="n">
-        <v>13.07</v>
-      </c>
-      <c r="H6" t="n">
-        <v>89.53</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>NSE:AXISBANK</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -685,17 +645,9 @@
       <c r="F7" t="n">
         <v>3.14</v>
       </c>
-      <c r="G7" t="n">
-        <v>59.07</v>
-      </c>
-      <c r="H7" t="n">
-        <v>12.94</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>NSE:INDUSINDBK</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -722,17 +674,9 @@
       <c r="F8" t="n">
         <v>3.1</v>
       </c>
-      <c r="G8" t="n">
-        <v>7.07</v>
-      </c>
-      <c r="H8" t="n">
-        <v>37.63</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>NSE:BANKBARODA</t>
-        </is>
-      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -759,17 +703,9 @@
       <c r="F9" t="n">
         <v>3.08</v>
       </c>
-      <c r="G9" t="n">
-        <v>12.86</v>
-      </c>
-      <c r="H9" t="n">
-        <v>16.34</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>NSE:FEDERALBNK</t>
-        </is>
-      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -796,17 +732,9 @@
       <c r="F10" t="n">
         <v>2.99</v>
       </c>
-      <c r="G10" t="n">
-        <v>42.22</v>
-      </c>
-      <c r="H10" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>NSE:IDFCFIRSTB</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -833,17 +761,9 @@
       <c r="F11" t="n">
         <v>2.71</v>
       </c>
-      <c r="G11" t="n">
-        <v>6.92</v>
-      </c>
-      <c r="H11" t="n">
-        <v>18.38</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>NSE:CANBK</t>
-        </is>
-      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -870,17 +790,9 @@
       <c r="F12" t="n">
         <v>2.67</v>
       </c>
-      <c r="G12" t="n">
-        <v>26.21</v>
-      </c>
-      <c r="H12" t="n">
-        <v>29.28</v>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>NSE:AUBANK</t>
-        </is>
-      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -907,17 +819,9 @@
       <c r="F13" t="n">
         <v>2.52</v>
       </c>
-      <c r="G13" t="n">
-        <v>7.95</v>
-      </c>
-      <c r="H13" t="n">
-        <v>14.63</v>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>NSE:PNB</t>
-        </is>
-      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix merge errors in join, create a standalone runner script
</commit_message>
<xml_diff>
--- a/off-disc/bank-nifty-ffat.xlsx
+++ b/off-disc/bank-nifty-ffat.xlsx
@@ -461,12 +461,12 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>eps</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>pe</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>eps</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -502,7 +502,11 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -531,7 +535,11 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -560,7 +568,11 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -589,7 +601,11 @@
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -618,7 +634,11 @@
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>AXISBANK</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -647,7 +667,11 @@
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>INDUSINDBK</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -676,7 +700,11 @@
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>BANKBARODA</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -705,7 +733,11 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>FEDERALBNK</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -734,7 +766,11 @@
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>IDFCFIRSTB</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -763,7 +799,11 @@
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>CANBK</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -792,7 +832,11 @@
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>AUBANK</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -821,7 +865,11 @@
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>PNB</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>